<commit_message>
Updated SYDEC with new data center BTM gas data
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
+++ b/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\bldgs\SYDEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\bldgs\SYDEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFE0D22-2FF1-40A2-B102-F217EB005F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A578AD3-D476-4117-8DCD-4CF8A8F12148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24900" yWindow="3810" windowWidth="21600" windowHeight="12585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -25,21 +25,19 @@
     <sheet name="Calcs&gt;" sheetId="8" r:id="rId10"/>
     <sheet name="Calculations" sheetId="9" r:id="rId11"/>
     <sheet name="Inflation Reduction Act" sheetId="10" r:id="rId12"/>
-    <sheet name="BDESC-urban-residential" sheetId="11" r:id="rId13"/>
-    <sheet name="BDESC-rural-residential" sheetId="12" r:id="rId14"/>
-    <sheet name="BDESC-commercial" sheetId="13" r:id="rId15"/>
-    <sheet name="SYDEC" sheetId="18" r:id="rId16"/>
+    <sheet name="Data Center Gas" sheetId="18" r:id="rId13"/>
+    <sheet name="BDESC-urban-residential" sheetId="11" r:id="rId14"/>
+    <sheet name="BDESC-rural-residential" sheetId="12" r:id="rId15"/>
+    <sheet name="BDESC-commercial" sheetId="13" r:id="rId16"/>
+    <sheet name="SYDEC" sheetId="19" r:id="rId17"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId17"/>
-  </externalReferences>
   <definedNames>
-    <definedName name="billion_kw_to_MW" localSheetId="15">#REF!</definedName>
-    <definedName name="billion_kw_to_MW">About!$B$28</definedName>
+    <definedName name="billion_kw_to_MW" localSheetId="16">#REF!</definedName>
+    <definedName name="billion_kw_to_MW">About!$B$35</definedName>
     <definedName name="Fraction_coal">#REF!</definedName>
     <definedName name="gal_per_barrel">#REF!</definedName>
-    <definedName name="gigwatt_to_megawatt" localSheetId="15">#REF!</definedName>
-    <definedName name="gigwatt_to_megawatt">About!$B$29</definedName>
+    <definedName name="gigwatt_to_megawatt" localSheetId="16">#REF!</definedName>
+    <definedName name="gigwatt_to_megawatt">About!$B$36</definedName>
     <definedName name="IQ_CH">110000</definedName>
     <definedName name="IQ_CQ">5000</definedName>
     <definedName name="IQ_CY">10000</definedName>
@@ -66,10 +64,10 @@
     <definedName name="IQ_WEEK">50000</definedName>
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
-    <definedName name="Percent_rural" localSheetId="15">#REF!</definedName>
-    <definedName name="Percent_rural">About!$A$26</definedName>
-    <definedName name="Percent_urban" localSheetId="15">#REF!</definedName>
-    <definedName name="Percent_Urban">About!$A$25</definedName>
+    <definedName name="Percent_rural" localSheetId="16">#REF!</definedName>
+    <definedName name="Percent_rural">About!$A$33</definedName>
+    <definedName name="Percent_urban" localSheetId="16">#REF!</definedName>
+    <definedName name="Percent_Urban">About!$A$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'EPM Table_6_02_B'!$1:$4</definedName>
     <definedName name="quadrillion">#REF!</definedName>
     <definedName name="Table4">#REF!</definedName>
@@ -103,7 +101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2053" uniqueCount="980">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2078" uniqueCount="1001">
   <si>
     <t>Sources:</t>
   </si>
@@ -3052,6 +3050,80 @@
   </si>
   <si>
     <t>rural</t>
+  </si>
+  <si>
+    <t>Behind-the-meter Data Center Gas Plants</t>
+  </si>
+  <si>
+    <r>
+      <t>Table 3.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13.5"/>
+        <color rgb="FF161400"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> Overall Behind-the-Meter Effective Capacity Growth by Region Out to 2030 (GW)</t>
+    </r>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Forecast</t>
+  </si>
+  <si>
+    <t>ISO regions</t>
+  </si>
+  <si>
+    <t>CAISO</t>
+  </si>
+  <si>
+    <t>ERCOT</t>
+  </si>
+  <si>
+    <t>NE-ISO</t>
+  </si>
+  <si>
+    <t>MISO</t>
+  </si>
+  <si>
+    <t>NY-ISO</t>
+  </si>
+  <si>
+    <t>PJM</t>
+  </si>
+  <si>
+    <t>SPP</t>
+  </si>
+  <si>
+    <t>Non-ISO regions</t>
+  </si>
+  <si>
+    <t>Annual incremental</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>RAND has estimated the behind the meter capacity to support data centers through 2030.</t>
+  </si>
+  <si>
+    <t>We assume 100% of this gas.</t>
+  </si>
+  <si>
+    <t>We add this forecasted capacity to AEO forecasts, which isn't capturing this trend</t>
+  </si>
+  <si>
+    <t>RAND</t>
+  </si>
+  <si>
+    <t>https://www.rand.org/pubs/research_briefs/RBA3845-1.html</t>
+  </si>
+  <si>
+    <t>How Much More Power Can the U.S. Grid Provide for AI?</t>
   </si>
   <si>
     <t>urban residential</t>
@@ -3076,7 +3148,7 @@
     <numFmt numFmtId="168" formatCode="0.00000000000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3261,8 +3333,34 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="13.5"/>
+      <color rgb="FF161400"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color rgb="FF2D2B19"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF2D2B19"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF2D2B19"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3372,12 +3470,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -3554,6 +3658,94 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF2D2B19"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD0D0CC"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF2D2B19"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD0D0CC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD0D0CC"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color rgb="FF2D2B19"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color rgb="FF2D2B19"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFD0D0CC"/>
+      </right>
+      <top style="thick">
+        <color rgb="FF2D2B19"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFD0D0CC"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color rgb="FF2D2B19"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFD0D0CC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3589,7 +3781,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3718,11 +3910,27 @@
     <xf numFmtId="0" fontId="24" fillId="18" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -3730,7 +3938,13 @@
     <xf numFmtId="0" fontId="25" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3753,11 +3967,38 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="20">
     <cellStyle name="60% - Accent1 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
@@ -11268,48 +11509,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="About"/>
-      <sheetName val="Source Data&gt;"/>
-      <sheetName val="AEO25_Table_21._Residential"/>
-      <sheetName val="AEO25_Table_22._Commercial"/>
-      <sheetName val="RECS HC2.1"/>
-      <sheetName val="AEO26_Table_21._Residential"/>
-      <sheetName val="AEO26_Table_22._Commercial"/>
-      <sheetName val="Calcs&gt;"/>
-      <sheetName val="Calculations"/>
-      <sheetName val="Inflation Reduction Act"/>
-      <sheetName val="BDESC-urban-residential"/>
-      <sheetName val="BDESC-rural-residential"/>
-      <sheetName val="BDESC-commercial"/>
-      <sheetName val="SYDEC"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -11597,7 +11796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51.85546875" customWidth="1"/>
@@ -11608,7 +11807,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>979</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -11707,7 +11906,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B17" s="18" t="s">
         <v>8</v>
       </c>
@@ -11715,159 +11914,184 @@
         <v>962</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B22" s="2">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="18" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="8">
         <f>'RECS HC2.1'!B24/SUM('RECS HC2.1'!B24,'RECS HC2.1'!B27)</f>
         <v>0.81308184246741677</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B32" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="8">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="8">
         <f>'RECS HC2.1'!B27/SUM('RECS HC2.1'!B24,'RECS HC2.1'!B27)</f>
         <v>0.18691815753258317</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B33" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B28">
+      <c r="B35">
         <f>10^6</f>
         <v>1000000</v>
       </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="13"/>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="C35" s="11"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="13"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>18</v>
       </c>
-      <c r="B29">
+      <c r="B36">
         <v>1000</v>
       </c>
-      <c r="F29" s="13"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+      <c r="F36" s="13"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
         <v>972</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>971</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>968</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B41" t="s">
         <v>969</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42">
         <f>AEO26_Table_21._Residential!E77</f>
         <v>44.365597000000001</v>
       </c>
-      <c r="B35">
+      <c r="B42">
         <f>'STEO Feb26'!B40</f>
         <v>40.4</v>
       </c>
-      <c r="C35">
-        <f>A35-B35</f>
+      <c r="C42">
+        <f>A42-B42</f>
         <v>3.9655970000000025</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D42" t="s">
         <v>974</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43">
         <f>AEO26_Table_22._Commercial!E61</f>
         <v>33.559604999999998</v>
       </c>
-      <c r="B36">
+      <c r="B43">
         <f>SUM('STEO Feb26'!B41:B42)</f>
         <v>18.8</v>
       </c>
-      <c r="C36" s="1">
-        <f>11.6-C35</f>
+      <c r="C43" s="1">
+        <f>11.6-C42</f>
         <v>7.6344029999999972</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D43" t="s">
         <v>973</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B38" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B45" t="s">
         <v>970</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="55">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="55">
         <v>36072.861350926898</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B46" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="1">
-        <f>$C$35*A39/SUM($A$39:$A$40)</f>
+      <c r="C46" s="1">
+        <f>$C$42*A46/SUM($A$46:$A$47)</f>
         <v>3.2243549152432633</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D46" t="s">
         <v>975</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="55">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="55">
         <v>8292.7356490730999</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B47" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="1">
-        <f>$C$35*A40/SUM($A$39:$A$40)</f>
+      <c r="C47" s="1">
+        <f>$C$42*A47/SUM($A$46:$A$47)</f>
         <v>0.74124208475673992</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D47" t="s">
         <v>976</v>
       </c>
     </row>
@@ -12210,111 +12434,111 @@
         <v>529</v>
       </c>
       <c r="D6">
-        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B6,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B6,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$32*About!$B$35</f>
         <v>5555.7882295798581</v>
       </c>
       <c r="E6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>1627.7898486197685</v>
       </c>
       <c r="F6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>3557.2330607949489</v>
       </c>
       <c r="G6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>5437.8913624220841</v>
       </c>
       <c r="H6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>5479.358536387922</v>
       </c>
       <c r="I6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>5521.6387921962278</v>
       </c>
       <c r="J6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>8143.014652311178</v>
       </c>
       <c r="K6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>11642.518902290942</v>
       </c>
       <c r="L6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>15250.976119161336</v>
       </c>
       <c r="M6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>18060.986966728731</v>
       </c>
       <c r="N6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21580.818262770175</v>
       </c>
       <c r="O6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21622.285436736012</v>
       </c>
       <c r="P6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21663.752610701853</v>
       </c>
       <c r="Q6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21706.032866510159</v>
       </c>
       <c r="R6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21747.500040475996</v>
       </c>
       <c r="S6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21789.780296284302</v>
       </c>
       <c r="T6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21835.312879462479</v>
       </c>
       <c r="U6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21887.350117380389</v>
       </c>
       <c r="V6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>21954.022828462723</v>
       </c>
       <c r="W6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>22048.340322188938</v>
       </c>
       <c r="X6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>22197.947381202943</v>
       </c>
       <c r="Y6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>22450.815834210316</v>
       </c>
       <c r="Z6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>22894.75852019752</v>
       </c>
       <c r="AA6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>23341.140451712134</v>
       </c>
       <c r="AB6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>23789.148546911678</v>
       </c>
       <c r="AC6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>24239.595887638628</v>
       </c>
       <c r="AD6">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A6,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>24694.108637577912</v>
       </c>
     </row>
@@ -12501,111 +12725,111 @@
         <v>533</v>
       </c>
       <c r="D9">
-        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B9,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B9,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$32*About!$B$35</f>
         <v>300368.69424431311</v>
       </c>
       <c r="E9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>140072.86132923176</v>
       </c>
       <c r="F9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>140198.07593297173</v>
       </c>
       <c r="G9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>140350.9353193556</v>
       </c>
       <c r="H9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>140502.16854205454</v>
       </c>
       <c r="I9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>140746.90617663725</v>
       </c>
       <c r="J9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>141171.33489840524</v>
       </c>
       <c r="K9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>141941.32340322188</v>
       </c>
       <c r="L9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>143138.99295717638</v>
       </c>
       <c r="M9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>144978.99716668014</v>
       </c>
       <c r="N9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>147506.86861491136</v>
       </c>
       <c r="O9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>150522.589168623</v>
       </c>
       <c r="P9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>153902.57038776006</v>
       </c>
       <c r="Q9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>157645.18610863757</v>
       </c>
       <c r="R9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>161573.18448959765</v>
       </c>
       <c r="S9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>165598.75269165382</v>
       </c>
       <c r="T9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>169864.18003723791</v>
       </c>
       <c r="U9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>174618.26957014488</v>
       </c>
       <c r="V9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>179692.71334898405</v>
       </c>
       <c r="W9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>184928.14733263175</v>
       </c>
       <c r="X9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>190289.60900186186</v>
       </c>
       <c r="Y9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>195821.81785801018</v>
       </c>
       <c r="Z9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>201816.67028252245</v>
       </c>
       <c r="AA9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>208040.81178661055</v>
       </c>
       <c r="AB9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>215123.56771634417</v>
       </c>
       <c r="AC9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>222286.00566663966</v>
       </c>
       <c r="AD9">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A9,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>229521.62098275719</v>
       </c>
     </row>
@@ -12620,111 +12844,111 @@
         <v>535</v>
       </c>
       <c r="D10">
-        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B10,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B10,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$32*About!$B$35</f>
         <v>50978364.686796732</v>
       </c>
       <c r="E10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>53470950.009228528</v>
       </c>
       <c r="F10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>56521290.774710603</v>
       </c>
       <c r="G10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>59964463.088480517</v>
       </c>
       <c r="H10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>63515989.127823189</v>
       </c>
       <c r="I10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>66825908.71075853</v>
       </c>
       <c r="J10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>70302740.173561066</v>
       </c>
       <c r="K10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>74066152.901805222</v>
       </c>
       <c r="L10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>77813083.648020715</v>
       </c>
       <c r="M10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>81739216.006152347</v>
       </c>
       <c r="N10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>85899672.046628341</v>
       </c>
       <c r="O10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>90335556.308912814</v>
       </c>
       <c r="P10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>94982501.982028648</v>
       </c>
       <c r="Q10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>99960122.34890309</v>
       </c>
       <c r="R10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>105171992.40767422</v>
       </c>
       <c r="S10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>110663048.75252973</v>
       </c>
       <c r="T10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>116346805.49405001</v>
       </c>
       <c r="U10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>122255072.83315793</v>
       </c>
       <c r="V10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>128329093.41050757</v>
       </c>
       <c r="W10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>134590739.12766129</v>
       </c>
       <c r="X10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>141094736.08419007</v>
       </c>
       <c r="Y10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>147745429.26673684</v>
       </c>
       <c r="Z10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>154590957.18578482</v>
       </c>
       <c r="AA10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>161636864.24641788</v>
       </c>
       <c r="AB10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>168976932.12142801</v>
       </c>
       <c r="AC10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>176433189.3917267</v>
       </c>
       <c r="AD10">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A10,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$35</f>
         <v>184157193.69966808</v>
       </c>
     </row>
@@ -13776,111 +14000,111 @@
         <v>529</v>
       </c>
       <c r="D25">
-        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B25,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B25,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$33*About!$B$35</f>
         <v>1277.2117704201407</v>
       </c>
       <c r="E25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>374.21015138023148</v>
       </c>
       <c r="F25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>817.76693920505147</v>
       </c>
       <c r="G25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>1250.1086375779162</v>
       </c>
       <c r="H25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>1259.641463612078</v>
       </c>
       <c r="I25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>1269.3612078037722</v>
       </c>
       <c r="J25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>1871.9853476888204</v>
       </c>
       <c r="K25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>2676.4810977090583</v>
       </c>
       <c r="L25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>3506.0238808386625</v>
       </c>
       <c r="M25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>4152.0130332712697</v>
       </c>
       <c r="N25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>4961.1817372298228</v>
       </c>
       <c r="O25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>4970.714563263984</v>
       </c>
       <c r="P25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>4980.2473892981461</v>
       </c>
       <c r="Q25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>4989.9671334898403</v>
       </c>
       <c r="R25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>4999.4999595240024</v>
       </c>
       <c r="S25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5009.2197037156966</v>
       </c>
       <c r="T25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5019.687120537521</v>
       </c>
       <c r="U25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5031.6498826196057</v>
       </c>
       <c r="V25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5046.977171537279</v>
       </c>
       <c r="W25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5068.6596778110579</v>
       </c>
       <c r="X25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5103.0526187970527</v>
       </c>
       <c r="Y25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5161.1841657896866</v>
       </c>
       <c r="Z25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5263.2414798024765</v>
       </c>
       <c r="AA25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5365.8595482878654</v>
       </c>
       <c r="AB25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5468.8514530883176</v>
       </c>
       <c r="AC25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5572.4041123613697</v>
       </c>
       <c r="AD25">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A25,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>5676.8913624220831</v>
       </c>
     </row>
@@ -14067,111 +14291,111 @@
         <v>533</v>
       </c>
       <c r="D28">
-        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B28,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B28,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$33*About!$B$35</f>
         <v>69051.305755686888</v>
       </c>
       <c r="E28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32201.138670768236</v>
       </c>
       <c r="F28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32229.924067028252</v>
       </c>
       <c r="G28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32265.064680644376</v>
       </c>
       <c r="H28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32299.831457945438</v>
       </c>
       <c r="I28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32356.093823362749</v>
       </c>
       <c r="J28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32453.665101594754</v>
       </c>
       <c r="K28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32630.67659677811</v>
       </c>
       <c r="L28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32906.007042823607</v>
       </c>
       <c r="M28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>33329.002833319842</v>
       </c>
       <c r="N28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>33910.131385088636</v>
       </c>
       <c r="O28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>34603.410831376998</v>
       </c>
       <c r="P28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>35380.429612239946</v>
       </c>
       <c r="Q28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>36240.813891362428</v>
       </c>
       <c r="R28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>37143.815510402332</v>
       </c>
       <c r="S28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>38069.247308346145</v>
       </c>
       <c r="T28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>39049.819962762078</v>
       </c>
       <c r="U28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>40142.730429855095</v>
       </c>
       <c r="V28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>41309.286651015951</v>
       </c>
       <c r="W28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>42512.85266736825</v>
       </c>
       <c r="X28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>43745.3909981381</v>
       </c>
       <c r="Y28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>45017.182141989797</v>
       </c>
       <c r="Z28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>46395.329717477536</v>
       </c>
       <c r="AA28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>47826.188213389454</v>
       </c>
       <c r="AB28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>49454.432283655784</v>
       </c>
       <c r="AC28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>51100.994333360315</v>
       </c>
       <c r="AD28">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A28,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>52764.379017242769</v>
       </c>
     </row>
@@ -14186,111 +14410,111 @@
         <v>535</v>
       </c>
       <c r="D29">
-        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B29,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$82:$AG$93,MATCH($B29,AEO25_Table_21._Residential!$B$82:$B$93,0),MATCH(D$4,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$33*About!$B$35</f>
         <v>11719339.313203271</v>
       </c>
       <c r="E29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>12292355.990771472</v>
       </c>
       <c r="F29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>12993594.225289404</v>
       </c>
       <c r="G29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>13785139.911519468</v>
       </c>
       <c r="H29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>14601594.872176796</v>
       </c>
       <c r="I29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>15362507.28924148</v>
       </c>
       <c r="J29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>16161790.826438921</v>
       </c>
       <c r="K29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>17026956.098194771</v>
       </c>
       <c r="L29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>17888332.351979274</v>
       </c>
       <c r="M29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>18790904.993847646</v>
       </c>
       <c r="N29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>19747345.953371648</v>
       </c>
       <c r="O29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>20767104.691087183</v>
       </c>
       <c r="P29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>21835384.017971344</v>
       </c>
       <c r="Q29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>22979681.651096895</v>
       </c>
       <c r="R29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>24177830.592325747</v>
       </c>
       <c r="S29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>25440161.247470248</v>
       </c>
       <c r="T29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>26746791.505949967</v>
       </c>
       <c r="U29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>28105034.166842062</v>
       </c>
       <c r="V29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>29501381.589492433</v>
       </c>
       <c r="W29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>30940861.872338701</v>
       </c>
       <c r="X29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>32436055.915809922</v>
       </c>
       <c r="Y29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>33964973.73326318</v>
       </c>
       <c r="Z29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>35538681.814215168</v>
       </c>
       <c r="AA29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>37158454.753582127</v>
       </c>
       <c r="AB29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>38845851.87857201</v>
       </c>
       <c r="AC29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>40559959.60827329</v>
       </c>
       <c r="AD29">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$28</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A29,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$4,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$35</f>
         <v>42335619.300331905</v>
       </c>
     </row>
@@ -15389,111 +15613,111 @@
         <v>529</v>
       </c>
       <c r="D44">
-        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B44,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B44,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$32*About!$B$36</f>
         <v>1.4025661782562939</v>
       </c>
       <c r="E44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>0.41060633044604544</v>
       </c>
       <c r="F44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>0.89845543592649557</v>
       </c>
       <c r="G44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>1.3732952319274669</v>
       </c>
       <c r="H44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>1.3838652958795432</v>
       </c>
       <c r="I44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>1.3944353598316197</v>
       </c>
       <c r="J44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>2.0562839796000971</v>
       </c>
       <c r="K44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>2.9401039423621791</v>
       </c>
       <c r="L44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>3.8515686877681534</v>
       </c>
       <c r="M44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>4.5605760543997409</v>
       </c>
       <c r="N44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.449274508216627</v>
       </c>
       <c r="O44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.459844572168703</v>
       </c>
       <c r="P44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.4704146361207799</v>
       </c>
       <c r="Q44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.480984700072856</v>
       </c>
       <c r="R44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.4915547640249329</v>
       </c>
       <c r="S44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.5029379098194759</v>
       </c>
       <c r="T44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.5143210556140208</v>
       </c>
       <c r="U44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.5273303650934995</v>
       </c>
       <c r="V44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.5444050837853149</v>
       </c>
       <c r="W44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.5679844572168697</v>
       </c>
       <c r="X44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.6053862219703712</v>
       </c>
       <c r="Y44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.6696196875252971</v>
       </c>
       <c r="Z44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.7818249817858005</v>
       </c>
       <c r="AA44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>5.8940302760463048</v>
       </c>
       <c r="AB44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>6.0070486521492752</v>
       </c>
       <c r="AC44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>6.1208801100947134</v>
       </c>
       <c r="AD44">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A44,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>6.2355246498826196</v>
       </c>
     </row>
@@ -15680,111 +15904,111 @@
         <v>533</v>
       </c>
       <c r="D47">
-        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B47,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B47,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$32*About!$B$36</f>
         <v>250.57474912976602</v>
       </c>
       <c r="E47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>131.09481162470655</v>
       </c>
       <c r="F47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>131.20376459159718</v>
       </c>
       <c r="G47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>131.33711001376184</v>
       </c>
       <c r="H47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>131.46882927224155</v>
       </c>
       <c r="I47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>131.68185671496801</v>
       </c>
       <c r="J47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>132.05262203513317</v>
       </c>
       <c r="K47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>132.72666688253864</v>
       </c>
       <c r="L47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>133.77960786853396</v>
       </c>
       <c r="M47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>135.40658463531125</v>
       </c>
       <c r="N47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>137.65150360236379</v>
       </c>
       <c r="O47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>140.33792600987613</v>
       </c>
       <c r="P47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>143.35527272727273</v>
       </c>
       <c r="Q47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>146.70191759086862</v>
       </c>
       <c r="R47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>150.2176834776977</v>
       </c>
       <c r="S47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>153.8212622035133</v>
       </c>
       <c r="T47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>157.64274686311018</v>
       </c>
       <c r="U47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>161.90654804500929</v>
       </c>
       <c r="V47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>166.46143252651177</v>
       </c>
       <c r="W47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>171.16429790334331</v>
       </c>
       <c r="X47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>175.98343398364767</v>
       </c>
       <c r="Y47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>180.96112102323323</v>
       </c>
       <c r="Z47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>186.38193766696349</v>
       </c>
       <c r="AA47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>192.00683785315306</v>
       </c>
       <c r="AB47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>198.43587598154292</v>
       </c>
       <c r="AC47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>204.93646531206994</v>
       </c>
       <c r="AD47">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A47,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>211.50616659920667</v>
       </c>
     </row>
@@ -15799,111 +16023,111 @@
         <v>535</v>
       </c>
       <c r="D48">
-        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B48,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B48,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$32*About!$B$36</f>
         <v>33586.644085485314</v>
       </c>
       <c r="E48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>36072.861350926898</v>
       </c>
       <c r="F48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>38259.984834453164</v>
       </c>
       <c r="G48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>40727.440236379822</v>
       </c>
       <c r="H48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>43279.974083056746</v>
       </c>
       <c r="I48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>45677.105223346553</v>
       </c>
       <c r="J48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>48200.653515421349</v>
       </c>
       <c r="K48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>50934.882696025255</v>
       </c>
       <c r="L48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>53663.724396340971</v>
       </c>
       <c r="M48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>56531.886044199789</v>
       </c>
       <c r="N48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>59575.347324212737</v>
       </c>
       <c r="O48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>62828.816260989224</v>
       </c>
       <c r="P48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>66242.132209503761</v>
       </c>
       <c r="Q48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>69907.185614182774</v>
       </c>
       <c r="R48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>73746.942662025409</v>
       </c>
       <c r="S48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>77794.55432591273</v>
       </c>
       <c r="T48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>81990.716855500679</v>
       </c>
       <c r="U48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>86364.605253460701</v>
       </c>
       <c r="V48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>90868.614390998133</v>
       </c>
       <c r="W48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>95514.394104751875</v>
       </c>
       <c r="X48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>100341.03086505302</v>
       </c>
       <c r="Y48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>105287.69639310289</v>
       </c>
       <c r="Z48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>110385.40081729133</v>
       </c>
       <c r="AA48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>115640.48292366226</v>
       </c>
       <c r="AB48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>121126.73883331985</v>
       </c>
       <c r="AC48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>126714.16976896301</v>
       </c>
       <c r="AD48">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$25*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A48,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$32*About!$B$36</f>
         <v>132502.56445203593</v>
       </c>
     </row>
@@ -16955,111 +17179,111 @@
         <v>529</v>
       </c>
       <c r="D63">
-        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B63,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B63,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$33*About!$B$36</f>
         <v>0.32243382174370594</v>
       </c>
       <c r="E63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>9.4393669553954507E-2</v>
       </c>
       <c r="F63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.20654456407350441</v>
       </c>
       <c r="G63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.31570476807253295</v>
       </c>
       <c r="H63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.31813470412045658</v>
       </c>
       <c r="I63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.32056464016838015</v>
       </c>
       <c r="J63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.47271602039990285</v>
       </c>
       <c r="K63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.67589605763782079</v>
       </c>
       <c r="L63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>0.88543131223184646</v>
       </c>
       <c r="M63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.0484239456002591</v>
       </c>
       <c r="N63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2527254917833723</v>
       </c>
       <c r="O63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.255155427831296</v>
       </c>
       <c r="P63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2575853638792196</v>
       </c>
       <c r="Q63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2600152999271432</v>
       </c>
       <c r="R63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2624452359750666</v>
       </c>
       <c r="S63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.265062090180523</v>
       </c>
       <c r="T63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2676789443859791</v>
       </c>
       <c r="U63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2706696349065005</v>
       </c>
       <c r="V63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2745949162146848</v>
       </c>
       <c r="W63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2800155427831297</v>
       </c>
       <c r="X63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.2886137780296285</v>
       </c>
       <c r="Y63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.3033803124747023</v>
       </c>
       <c r="Z63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.329175018214199</v>
       </c>
       <c r="AA63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.3549697239536955</v>
       </c>
       <c r="AB63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.3809513478507245</v>
       </c>
       <c r="AC63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.4071198899052861</v>
       </c>
       <c r="AD63">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A63,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>1.4334753501173803</v>
       </c>
     </row>
@@ -17246,111 +17470,111 @@
         <v>533</v>
       </c>
       <c r="D66">
-        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B66,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B66,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$33*About!$B$36</f>
         <v>57.60425087023394</v>
       </c>
       <c r="E66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.137188375293448</v>
       </c>
       <c r="F66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.162235408402818</v>
       </c>
       <c r="G66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.192889986238161</v>
       </c>
       <c r="H66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.223170727758436</v>
       </c>
       <c r="I66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.272143285031973</v>
       </c>
       <c r="J66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.357377964866835</v>
       </c>
       <c r="K66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.512333117461345</v>
       </c>
       <c r="L66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30.754392131466041</v>
       </c>
       <c r="M66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>31.128415364688738</v>
       </c>
       <c r="N66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>31.644496397636203</v>
       </c>
       <c r="O66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>32.262073990123852</v>
       </c>
       <c r="P66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>32.955727272727266</v>
       </c>
       <c r="Q66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>33.725082409131382</v>
       </c>
       <c r="R66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>34.533316522302272</v>
       </c>
       <c r="S66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>35.361737796486679</v>
       </c>
       <c r="T66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>36.240253136889827</v>
       </c>
       <c r="U66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>37.220451954990693</v>
       </c>
       <c r="V66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>38.267567473488214</v>
       </c>
       <c r="W66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>39.34870209665668</v>
       </c>
       <c r="X66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>40.456566016352298</v>
       </c>
       <c r="Y66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>41.600878976766779</v>
       </c>
       <c r="Z66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>42.847062333036504</v>
       </c>
       <c r="AA66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>44.140162146846919</v>
       </c>
       <c r="AB66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>45.618124018457053</v>
       </c>
       <c r="AC66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>47.112534687930058</v>
       </c>
       <c r="AD66">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A66,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>48.622833400793326</v>
       </c>
     </row>
@@ -17365,111 +17589,111 @@
         <v>535</v>
       </c>
       <c r="D67">
-        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B67,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO25_Table_21._Residential!$F$77:$AG$80,MATCH($B67,AEO25_Table_21._Residential!$B$77:$B$80,0),MATCH(D$42,AEO25_Table_21._Residential!$F$5:$AG$5,0))*About!$A$33*About!$B$36</f>
         <v>7721.182914514693</v>
       </c>
       <c r="E67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(E$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>8292.7356490730999</v>
       </c>
       <c r="F67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(F$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>8795.5301655468302</v>
       </c>
       <c r="G67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(G$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>9362.7697636201738</v>
       </c>
       <c r="H67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(H$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>9949.5679169432515</v>
       </c>
       <c r="I67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(I$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>10500.640776653445</v>
       </c>
       <c r="J67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(J$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>11080.775484578644</v>
       </c>
       <c r="K67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(K$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>11709.343303974743</v>
       </c>
       <c r="L67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(L$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>12336.67260365903</v>
       </c>
       <c r="M67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(M$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>12996.02995580021</v>
       </c>
       <c r="N67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(N$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>13695.686675787258</v>
       </c>
       <c r="O67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(O$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>14443.621739010765</v>
       </c>
       <c r="P67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(P$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>15228.303790496237</v>
       </c>
       <c r="Q67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Q$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>16070.857385817209</v>
       </c>
       <c r="R67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(R$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>16953.57333797458</v>
       </c>
       <c r="S67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(S$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>17884.072674087267</v>
       </c>
       <c r="T67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(T$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>18848.722144499312</v>
       </c>
       <c r="U67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(U$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>19854.228746539302</v>
       </c>
       <c r="V67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(V$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>20889.648609001859</v>
       </c>
       <c r="W67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(W$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>21957.659895248118</v>
       </c>
       <c r="X67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(X$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>23067.248134946974</v>
       </c>
       <c r="Y67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Y$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>24204.429606897113</v>
       </c>
       <c r="Z67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(Z$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>25376.333182708651</v>
       </c>
       <c r="AA67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AA$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>26584.416076337729</v>
       </c>
       <c r="AB67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AB$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>27845.643166680158</v>
       </c>
       <c r="AC67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AC$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>29130.129231036997</v>
       </c>
       <c r="AD67">
-        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$26*About!$B$29</f>
+        <f>INDEX(AEO26_Table_21._Residential!$E$6:$AD$92,MATCH($A67,AEO26_Table_21._Residential!$B$6:$B$92,0),MATCH(AD$42,AEO26_Table_21._Residential!$E$5:$AD$5,0))*About!$A$33*About!$B$36</f>
         <v>30460.814547964055</v>
       </c>
     </row>
@@ -23426,6 +23650,779 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{858104B2-5734-4794-B2D1-CAE7717AD060}">
+  <dimension ref="B2:AC27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="17.25" x14ac:dyDescent="0.25">
+      <c r="B7" s="65" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="87"/>
+      <c r="C9" s="89" t="s">
+        <v>979</v>
+      </c>
+      <c r="D9" s="89"/>
+      <c r="E9" s="90"/>
+      <c r="F9" s="91" t="s">
+        <v>980</v>
+      </c>
+      <c r="G9" s="89"/>
+      <c r="H9" s="89"/>
+      <c r="I9" s="89"/>
+    </row>
+    <row r="10" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="88"/>
+      <c r="C10" s="66">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="66">
+        <v>2025</v>
+      </c>
+      <c r="E10" s="67">
+        <v>2026</v>
+      </c>
+      <c r="F10" s="66">
+        <v>2027</v>
+      </c>
+      <c r="G10" s="66">
+        <v>2028</v>
+      </c>
+      <c r="H10" s="66">
+        <v>2029</v>
+      </c>
+      <c r="I10" s="66">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="92" t="s">
+        <v>981</v>
+      </c>
+      <c r="C11" s="92"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="93"/>
+      <c r="F11" s="94"/>
+      <c r="G11" s="95"/>
+      <c r="H11" s="95"/>
+      <c r="I11" s="95"/>
+    </row>
+    <row r="12" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="68" t="s">
+        <v>982</v>
+      </c>
+      <c r="C12" s="69">
+        <v>3</v>
+      </c>
+      <c r="D12" s="69">
+        <v>3.1</v>
+      </c>
+      <c r="E12" s="70">
+        <v>3.2</v>
+      </c>
+      <c r="F12" s="69">
+        <v>3.3</v>
+      </c>
+      <c r="G12" s="69">
+        <v>3.4</v>
+      </c>
+      <c r="H12" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="I12" s="69">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="68" t="s">
+        <v>983</v>
+      </c>
+      <c r="C13" s="69">
+        <v>2</v>
+      </c>
+      <c r="D13" s="69">
+        <v>3.3</v>
+      </c>
+      <c r="E13" s="70">
+        <v>4.7</v>
+      </c>
+      <c r="F13" s="69">
+        <v>4.8</v>
+      </c>
+      <c r="G13" s="69">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H13" s="69">
+        <v>6.9</v>
+      </c>
+      <c r="I13" s="69">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="68" t="s">
+        <v>984</v>
+      </c>
+      <c r="C14" s="69">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="69">
+        <v>0.2</v>
+      </c>
+      <c r="E14" s="70">
+        <v>0.2</v>
+      </c>
+      <c r="F14" s="69">
+        <v>0.4</v>
+      </c>
+      <c r="G14" s="69">
+        <v>0.6</v>
+      </c>
+      <c r="H14" s="69">
+        <v>0.8</v>
+      </c>
+      <c r="I14" s="69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="68" t="s">
+        <v>985</v>
+      </c>
+      <c r="C15" s="69">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D15" s="69">
+        <v>2.5</v>
+      </c>
+      <c r="E15" s="70">
+        <v>2.9</v>
+      </c>
+      <c r="F15" s="69">
+        <v>3.9</v>
+      </c>
+      <c r="G15" s="69">
+        <v>5</v>
+      </c>
+      <c r="H15" s="69">
+        <v>8.1</v>
+      </c>
+      <c r="I15" s="69">
+        <v>11.2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="68" t="s">
+        <v>986</v>
+      </c>
+      <c r="C16" s="69">
+        <v>0.8</v>
+      </c>
+      <c r="D16" s="69">
+        <v>1.6</v>
+      </c>
+      <c r="E16" s="70">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="F16" s="69">
+        <v>2.6</v>
+      </c>
+      <c r="G16" s="69">
+        <v>2.8</v>
+      </c>
+      <c r="H16" s="69">
+        <v>3</v>
+      </c>
+      <c r="I16" s="69">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="68" t="s">
+        <v>987</v>
+      </c>
+      <c r="C17" s="69">
+        <v>0.9</v>
+      </c>
+      <c r="D17" s="69">
+        <v>1.8</v>
+      </c>
+      <c r="E17" s="70">
+        <v>2.6</v>
+      </c>
+      <c r="F17" s="69">
+        <v>2.9</v>
+      </c>
+      <c r="G17" s="69">
+        <v>3.2</v>
+      </c>
+      <c r="H17" s="69">
+        <v>3.9</v>
+      </c>
+      <c r="I17" s="69">
+        <v>4.7</v>
+      </c>
+    </row>
+    <row r="18" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="68" t="s">
+        <v>988</v>
+      </c>
+      <c r="C18" s="69">
+        <v>0.5</v>
+      </c>
+      <c r="D18" s="69">
+        <v>0.6</v>
+      </c>
+      <c r="E18" s="70">
+        <v>0.7</v>
+      </c>
+      <c r="F18" s="69">
+        <v>0.9</v>
+      </c>
+      <c r="G18" s="69">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H18" s="69">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I18" s="69">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="19" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="68" t="s">
+        <v>989</v>
+      </c>
+      <c r="C19" s="69">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D19" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="E19" s="70">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="F19" s="69">
+        <v>6</v>
+      </c>
+      <c r="G19" s="69">
+        <v>7.3</v>
+      </c>
+      <c r="H19" s="69">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="I19" s="69">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="68" t="s">
+        <v>990</v>
+      </c>
+      <c r="C20" s="69" t="s">
+        <v>991</v>
+      </c>
+      <c r="D20" s="69">
+        <v>4.7</v>
+      </c>
+      <c r="E20" s="70">
+        <v>4.7</v>
+      </c>
+      <c r="F20" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="G20" s="69">
+        <v>3.5</v>
+      </c>
+      <c r="H20" s="69">
+        <v>10</v>
+      </c>
+      <c r="I20" s="69">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="2:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="71" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="69">
+        <v>12</v>
+      </c>
+      <c r="D21" s="69">
+        <v>17</v>
+      </c>
+      <c r="E21" s="70">
+        <v>21</v>
+      </c>
+      <c r="F21" s="69">
+        <v>25</v>
+      </c>
+      <c r="G21" s="69">
+        <v>29</v>
+      </c>
+      <c r="H21" s="69">
+        <v>39</v>
+      </c>
+      <c r="I21" s="69">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="24" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="C24">
+        <v>2024</v>
+      </c>
+      <c r="D24">
+        <v>2025</v>
+      </c>
+      <c r="E24">
+        <v>2026</v>
+      </c>
+      <c r="F24">
+        <v>2027</v>
+      </c>
+      <c r="G24">
+        <v>2028</v>
+      </c>
+      <c r="H24">
+        <v>2029</v>
+      </c>
+      <c r="I24">
+        <v>2030</v>
+      </c>
+      <c r="J24">
+        <v>2031</v>
+      </c>
+      <c r="K24">
+        <v>2032</v>
+      </c>
+      <c r="L24">
+        <v>2033</v>
+      </c>
+      <c r="M24">
+        <v>2034</v>
+      </c>
+      <c r="N24">
+        <v>2035</v>
+      </c>
+      <c r="O24">
+        <v>2036</v>
+      </c>
+      <c r="P24">
+        <v>2037</v>
+      </c>
+      <c r="Q24">
+        <v>2038</v>
+      </c>
+      <c r="R24">
+        <v>2039</v>
+      </c>
+      <c r="S24">
+        <v>2040</v>
+      </c>
+      <c r="T24">
+        <v>2041</v>
+      </c>
+      <c r="U24">
+        <v>2042</v>
+      </c>
+      <c r="V24">
+        <v>2043</v>
+      </c>
+      <c r="W24">
+        <v>2044</v>
+      </c>
+      <c r="X24">
+        <v>2045</v>
+      </c>
+      <c r="Y24">
+        <v>2046</v>
+      </c>
+      <c r="Z24">
+        <v>2047</v>
+      </c>
+      <c r="AA24">
+        <v>2048</v>
+      </c>
+      <c r="AB24">
+        <v>2049</v>
+      </c>
+      <c r="AC24">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="25" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B25" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="C25">
+        <f>Calculations!D44</f>
+        <v>1.4025661782562939</v>
+      </c>
+      <c r="D25">
+        <f>Calculations!E44</f>
+        <v>0.41060633044604544</v>
+      </c>
+      <c r="E25">
+        <f>Calculations!F44</f>
+        <v>0.89845543592649557</v>
+      </c>
+      <c r="F25">
+        <f>Calculations!G44</f>
+        <v>1.3732952319274669</v>
+      </c>
+      <c r="G25">
+        <f>Calculations!H44</f>
+        <v>1.3838652958795432</v>
+      </c>
+      <c r="H25">
+        <f>Calculations!I44</f>
+        <v>1.3944353598316197</v>
+      </c>
+      <c r="I25">
+        <f>Calculations!J44</f>
+        <v>2.0562839796000971</v>
+      </c>
+      <c r="J25">
+        <f>Calculations!K44</f>
+        <v>2.9401039423621791</v>
+      </c>
+      <c r="K25">
+        <f>Calculations!L44</f>
+        <v>3.8515686877681534</v>
+      </c>
+      <c r="L25">
+        <f>Calculations!M44</f>
+        <v>4.5605760543997409</v>
+      </c>
+      <c r="M25">
+        <f>Calculations!N44</f>
+        <v>5.449274508216627</v>
+      </c>
+      <c r="N25">
+        <f>Calculations!O44</f>
+        <v>5.459844572168703</v>
+      </c>
+      <c r="O25">
+        <f>Calculations!P44</f>
+        <v>5.4704146361207799</v>
+      </c>
+      <c r="P25">
+        <f>Calculations!Q44</f>
+        <v>5.480984700072856</v>
+      </c>
+      <c r="Q25">
+        <f>Calculations!R44</f>
+        <v>5.4915547640249329</v>
+      </c>
+      <c r="R25">
+        <f>Calculations!S44</f>
+        <v>5.5029379098194759</v>
+      </c>
+      <c r="S25">
+        <f>Calculations!T44</f>
+        <v>5.5143210556140208</v>
+      </c>
+      <c r="T25">
+        <f>Calculations!U44</f>
+        <v>5.5273303650934995</v>
+      </c>
+      <c r="U25">
+        <f>Calculations!V44</f>
+        <v>5.5444050837853149</v>
+      </c>
+      <c r="V25">
+        <f>Calculations!W44</f>
+        <v>5.5679844572168697</v>
+      </c>
+      <c r="W25">
+        <f>Calculations!X44</f>
+        <v>5.6053862219703712</v>
+      </c>
+      <c r="X25">
+        <f>Calculations!Y44</f>
+        <v>5.6696196875252971</v>
+      </c>
+      <c r="Y25">
+        <f>Calculations!Z44</f>
+        <v>5.7818249817858005</v>
+      </c>
+      <c r="Z25">
+        <f>Calculations!AA44</f>
+        <v>5.8940302760463048</v>
+      </c>
+      <c r="AA25">
+        <f>Calculations!AB44</f>
+        <v>6.0070486521492752</v>
+      </c>
+      <c r="AB25">
+        <f>Calculations!AC44</f>
+        <v>6.1208801100947134</v>
+      </c>
+      <c r="AC25">
+        <f>Calculations!AD44</f>
+        <v>6.2355246498826196</v>
+      </c>
+    </row>
+    <row r="26" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B26" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="C26">
+        <f>Calculations!D63</f>
+        <v>0.32243382174370594</v>
+      </c>
+      <c r="D26">
+        <f>Calculations!E63</f>
+        <v>9.4393669553954507E-2</v>
+      </c>
+      <c r="E26">
+        <f>Calculations!F63</f>
+        <v>0.20654456407350441</v>
+      </c>
+      <c r="F26">
+        <f>Calculations!G63</f>
+        <v>0.31570476807253295</v>
+      </c>
+      <c r="G26">
+        <f>Calculations!H63</f>
+        <v>0.31813470412045658</v>
+      </c>
+      <c r="H26">
+        <f>Calculations!I63</f>
+        <v>0.32056464016838015</v>
+      </c>
+      <c r="I26">
+        <f>Calculations!J63</f>
+        <v>0.47271602039990285</v>
+      </c>
+      <c r="J26">
+        <f>Calculations!K63</f>
+        <v>0.67589605763782079</v>
+      </c>
+      <c r="K26">
+        <f>Calculations!L63</f>
+        <v>0.88543131223184646</v>
+      </c>
+      <c r="L26">
+        <f>Calculations!M63</f>
+        <v>1.0484239456002591</v>
+      </c>
+      <c r="M26">
+        <f>Calculations!N63</f>
+        <v>1.2527254917833723</v>
+      </c>
+      <c r="N26">
+        <f>Calculations!O63</f>
+        <v>1.255155427831296</v>
+      </c>
+      <c r="O26">
+        <f>Calculations!P63</f>
+        <v>1.2575853638792196</v>
+      </c>
+      <c r="P26">
+        <f>Calculations!Q63</f>
+        <v>1.2600152999271432</v>
+      </c>
+      <c r="Q26">
+        <f>Calculations!R63</f>
+        <v>1.2624452359750666</v>
+      </c>
+      <c r="R26">
+        <f>Calculations!S63</f>
+        <v>1.265062090180523</v>
+      </c>
+      <c r="S26">
+        <f>Calculations!T63</f>
+        <v>1.2676789443859791</v>
+      </c>
+      <c r="T26">
+        <f>Calculations!U63</f>
+        <v>1.2706696349065005</v>
+      </c>
+      <c r="U26">
+        <f>Calculations!V63</f>
+        <v>1.2745949162146848</v>
+      </c>
+      <c r="V26">
+        <f>Calculations!W63</f>
+        <v>1.2800155427831297</v>
+      </c>
+      <c r="W26">
+        <f>Calculations!X63</f>
+        <v>1.2886137780296285</v>
+      </c>
+      <c r="X26">
+        <f>Calculations!Y63</f>
+        <v>1.3033803124747023</v>
+      </c>
+      <c r="Y26">
+        <f>Calculations!Z63</f>
+        <v>1.329175018214199</v>
+      </c>
+      <c r="Z26">
+        <f>Calculations!AA63</f>
+        <v>1.3549697239536955</v>
+      </c>
+      <c r="AA26">
+        <f>Calculations!AB63</f>
+        <v>1.3809513478507245</v>
+      </c>
+      <c r="AB26">
+        <f>Calculations!AC63</f>
+        <v>1.4071198899052861</v>
+      </c>
+      <c r="AC26">
+        <f>Calculations!AD63</f>
+        <v>1.4334753501173803</v>
+      </c>
+    </row>
+    <row r="27" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B27" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C27">
+        <f>Calculations!D84+C21*1000</f>
+        <v>13468.725</v>
+      </c>
+      <c r="D27">
+        <f>Calculations!E84+D21*1000</f>
+        <v>18508.008000000002</v>
+      </c>
+      <c r="E27">
+        <f>Calculations!F84+E21*1000</f>
+        <v>22540.969000000001</v>
+      </c>
+      <c r="F27">
+        <f>Calculations!G84+F21*1000</f>
+        <v>26559.125</v>
+      </c>
+      <c r="G27">
+        <f>Calculations!H84+G21*1000</f>
+        <v>30576.868999999999</v>
+      </c>
+      <c r="H27">
+        <f>Calculations!I84+H21*1000</f>
+        <v>40595.394999999997</v>
+      </c>
+      <c r="I27">
+        <f>Calculations!J84+I21*1000</f>
+        <v>50615.290999999997</v>
+      </c>
+      <c r="J27">
+        <f>Calculations!K84+$I$21*1000</f>
+        <v>50634.760999999999</v>
+      </c>
+      <c r="K27">
+        <f>Calculations!L84+$I$21*1000</f>
+        <v>50655.343999999997</v>
+      </c>
+      <c r="L27">
+        <f>Calculations!M84+$I$21*1000</f>
+        <v>50676.552000000003</v>
+      </c>
+      <c r="M27">
+        <f>Calculations!N84+$I$21*1000</f>
+        <v>50700.095000000001</v>
+      </c>
+      <c r="N27">
+        <f>Calculations!O84+$I$21*1000</f>
+        <v>50722.014000000003</v>
+      </c>
+      <c r="O27">
+        <f>Calculations!P84+$I$21*1000</f>
+        <v>50744.811999999998</v>
+      </c>
+      <c r="P27">
+        <f>Calculations!Q84+$I$21*1000</f>
+        <v>50769.997000000003</v>
+      </c>
+      <c r="Q27">
+        <f>Calculations!R84+$I$21*1000</f>
+        <v>50793.459000000003</v>
+      </c>
+      <c r="R27">
+        <f>Calculations!S84+$I$21*1000</f>
+        <v>50816.315999999999</v>
+      </c>
+      <c r="S27">
+        <f>Calculations!T84+$I$21*1000</f>
+        <v>50838.228000000003</v>
+      </c>
+      <c r="T27">
+        <f>Calculations!U84+$I$21*1000</f>
+        <v>50858.498999999996</v>
+      </c>
+      <c r="U27">
+        <f>Calculations!V84+$I$21*1000</f>
+        <v>50881.084999999999</v>
+      </c>
+      <c r="V27">
+        <f>Calculations!W84+$I$21*1000</f>
+        <v>50901.161999999997</v>
+      </c>
+      <c r="W27">
+        <f>Calculations!X84+$I$21*1000</f>
+        <v>50921.178</v>
+      </c>
+      <c r="X27">
+        <f>Calculations!Y84+$I$21*1000</f>
+        <v>50940.084000000003</v>
+      </c>
+      <c r="Y27">
+        <f>Calculations!Z84+$I$21*1000</f>
+        <v>50959.432999999997</v>
+      </c>
+      <c r="Z27">
+        <f>Calculations!AA84+$I$21*1000</f>
+        <v>50979.940999999999</v>
+      </c>
+      <c r="AA27">
+        <f>Calculations!AB84+$I$21*1000</f>
+        <v>51000.097000000002</v>
+      </c>
+      <c r="AB27">
+        <f>Calculations!AC84+$I$21*1000</f>
+        <v>51019.017999999996</v>
+      </c>
+      <c r="AC27">
+        <f>Calculations!AD84+$I$21*1000</f>
+        <v>51039.06</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="F11:I11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -24100,111 +25097,111 @@
         <v>535</v>
       </c>
       <c r="B8" s="55">
-        <f>Calculations!D48-About!$C$39*1000</f>
+        <f>Calculations!D48-About!$C$46*1000</f>
         <v>30362.289170242049</v>
       </c>
       <c r="C8" s="55">
-        <f>Calculations!E48-About!$C$39*1000</f>
+        <f>Calculations!E48-About!$C$46*1000</f>
         <v>32848.506435683637</v>
       </c>
       <c r="D8" s="55">
-        <f>Calculations!F48-About!$C$39*1000</f>
+        <f>Calculations!F48-About!$C$46*1000</f>
         <v>35035.629919209903</v>
       </c>
       <c r="E8" s="55">
-        <f>Calculations!G48-About!$C$39*1000</f>
+        <f>Calculations!G48-About!$C$46*1000</f>
         <v>37503.085321136561</v>
       </c>
       <c r="F8" s="55">
-        <f>Calculations!H48-About!$C$39*1000</f>
+        <f>Calculations!H48-About!$C$46*1000</f>
         <v>40055.619167813486</v>
       </c>
       <c r="G8" s="55">
-        <f>Calculations!I48-About!$C$39*1000</f>
+        <f>Calculations!I48-About!$C$46*1000</f>
         <v>42452.750308103292</v>
       </c>
       <c r="H8" s="55">
-        <f>Calculations!J48-About!$C$39*1000</f>
+        <f>Calculations!J48-About!$C$46*1000</f>
         <v>44976.298600178088</v>
       </c>
       <c r="I8" s="55">
-        <f>Calculations!K48-About!$C$39*1000</f>
+        <f>Calculations!K48-About!$C$46*1000</f>
         <v>47710.527780781995</v>
       </c>
       <c r="J8" s="55">
-        <f>Calculations!L48-About!$C$39*1000</f>
+        <f>Calculations!L48-About!$C$46*1000</f>
         <v>50439.36948109771</v>
       </c>
       <c r="K8" s="55">
-        <f>Calculations!M48-About!$C$39*1000</f>
+        <f>Calculations!M48-About!$C$46*1000</f>
         <v>53307.531128956529</v>
       </c>
       <c r="L8" s="55">
-        <f>Calculations!N48-About!$C$39*1000</f>
+        <f>Calculations!N48-About!$C$46*1000</f>
         <v>56350.992408969476</v>
       </c>
       <c r="M8" s="55">
-        <f>Calculations!O48-About!$C$39*1000</f>
+        <f>Calculations!O48-About!$C$46*1000</f>
         <v>59604.461345745964</v>
       </c>
       <c r="N8" s="55">
-        <f>Calculations!P48-About!$C$39*1000</f>
+        <f>Calculations!P48-About!$C$46*1000</f>
         <v>63017.777294260501</v>
       </c>
       <c r="O8" s="55">
-        <f>Calculations!Q48-About!$C$39*1000</f>
+        <f>Calculations!Q48-About!$C$46*1000</f>
         <v>66682.830698939506</v>
       </c>
       <c r="P8" s="55">
-        <f>Calculations!R48-About!$C$39*1000</f>
+        <f>Calculations!R48-About!$C$46*1000</f>
         <v>70522.587746782141</v>
       </c>
       <c r="Q8" s="55">
-        <f>Calculations!S48-About!$C$39*1000</f>
+        <f>Calculations!S48-About!$C$46*1000</f>
         <v>74570.199410669462</v>
       </c>
       <c r="R8" s="55">
-        <f>Calculations!T48-About!$C$39*1000</f>
+        <f>Calculations!T48-About!$C$46*1000</f>
         <v>78766.361940257411</v>
       </c>
       <c r="S8" s="55">
-        <f>Calculations!U48-About!$C$39*1000</f>
+        <f>Calculations!U48-About!$C$46*1000</f>
         <v>83140.250338217433</v>
       </c>
       <c r="T8" s="55">
-        <f>Calculations!V48-About!$C$39*1000</f>
+        <f>Calculations!V48-About!$C$46*1000</f>
         <v>87644.259475754865</v>
       </c>
       <c r="U8" s="55">
-        <f>Calculations!W48-About!$C$39*1000</f>
+        <f>Calculations!W48-About!$C$46*1000</f>
         <v>92290.039189508607</v>
       </c>
       <c r="V8" s="55">
-        <f>Calculations!X48-About!$C$39*1000</f>
+        <f>Calculations!X48-About!$C$46*1000</f>
         <v>97116.675949809753</v>
       </c>
       <c r="W8" s="55">
-        <f>Calculations!Y48-About!$C$39*1000</f>
+        <f>Calculations!Y48-About!$C$46*1000</f>
         <v>102063.34147785962</v>
       </c>
       <c r="X8" s="55">
-        <f>Calculations!Z48-About!$C$39*1000</f>
+        <f>Calculations!Z48-About!$C$46*1000</f>
         <v>107161.04590204806</v>
       </c>
       <c r="Y8" s="55">
-        <f>Calculations!AA48-About!$C$39*1000</f>
+        <f>Calculations!AA48-About!$C$46*1000</f>
         <v>112416.12800841899</v>
       </c>
       <c r="Z8" s="55">
-        <f>Calculations!AB48-About!$C$39*1000</f>
+        <f>Calculations!AB48-About!$C$46*1000</f>
         <v>117902.38391807658</v>
       </c>
       <c r="AA8" s="55">
-        <f>Calculations!AC48-About!$C$39*1000</f>
+        <f>Calculations!AC48-About!$C$46*1000</f>
         <v>123489.81485371974</v>
       </c>
       <c r="AB8" s="55">
-        <f>Calculations!AD48-About!$C$39*1000</f>
+        <f>Calculations!AD48-About!$C$46*1000</f>
         <v>129278.20953679267</v>
       </c>
     </row>
@@ -25681,7 +26678,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -26435,111 +27432,111 @@
         <v>535</v>
       </c>
       <c r="B8">
-        <f>Calculations!D67-About!$C$40*1000</f>
+        <f>Calculations!D67-About!$C$47*1000</f>
         <v>6979.940829757953</v>
       </c>
       <c r="C8">
-        <f>Calculations!E67-About!$C$40*1000</f>
+        <f>Calculations!E67-About!$C$47*1000</f>
         <v>7551.4935643163599</v>
       </c>
       <c r="D8">
-        <f>Calculations!F67-About!$C$40*1000</f>
+        <f>Calculations!F67-About!$C$47*1000</f>
         <v>8054.2880807900901</v>
       </c>
       <c r="E8">
-        <f>Calculations!G67-About!$C$40*1000</f>
+        <f>Calculations!G67-About!$C$47*1000</f>
         <v>8621.5276788634346</v>
       </c>
       <c r="F8">
-        <f>Calculations!H67-About!$C$40*1000</f>
+        <f>Calculations!H67-About!$C$47*1000</f>
         <v>9208.3258321865123</v>
       </c>
       <c r="G8">
-        <f>Calculations!I67-About!$C$40*1000</f>
+        <f>Calculations!I67-About!$C$47*1000</f>
         <v>9759.3986918967057</v>
       </c>
       <c r="H8">
-        <f>Calculations!J67-About!$C$40*1000</f>
+        <f>Calculations!J67-About!$C$47*1000</f>
         <v>10339.533399821905</v>
       </c>
       <c r="I8">
-        <f>Calculations!K67-About!$C$40*1000</f>
+        <f>Calculations!K67-About!$C$47*1000</f>
         <v>10968.101219218004</v>
       </c>
       <c r="J8">
-        <f>Calculations!L67-About!$C$40*1000</f>
+        <f>Calculations!L67-About!$C$47*1000</f>
         <v>11595.430518902291</v>
       </c>
       <c r="K8">
-        <f>Calculations!M67-About!$C$40*1000</f>
+        <f>Calculations!M67-About!$C$47*1000</f>
         <v>12254.787871043471</v>
       </c>
       <c r="L8">
-        <f>Calculations!N67-About!$C$40*1000</f>
+        <f>Calculations!N67-About!$C$47*1000</f>
         <v>12954.444591030518</v>
       </c>
       <c r="M8">
-        <f>Calculations!O67-About!$C$40*1000</f>
+        <f>Calculations!O67-About!$C$47*1000</f>
         <v>13702.379654254026</v>
       </c>
       <c r="N8">
-        <f>Calculations!P67-About!$C$40*1000</f>
+        <f>Calculations!P67-About!$C$47*1000</f>
         <v>14487.061705739497</v>
       </c>
       <c r="O8">
-        <f>Calculations!Q67-About!$C$40*1000</f>
+        <f>Calculations!Q67-About!$C$47*1000</f>
         <v>15329.61530106047</v>
       </c>
       <c r="P8">
-        <f>Calculations!R67-About!$C$40*1000</f>
+        <f>Calculations!R67-About!$C$47*1000</f>
         <v>16212.331253217841</v>
       </c>
       <c r="Q8">
-        <f>Calculations!S67-About!$C$40*1000</f>
+        <f>Calculations!S67-About!$C$47*1000</f>
         <v>17142.830589330526</v>
       </c>
       <c r="R8">
-        <f>Calculations!T67-About!$C$40*1000</f>
+        <f>Calculations!T67-About!$C$47*1000</f>
         <v>18107.480059742571</v>
       </c>
       <c r="S8">
-        <f>Calculations!U67-About!$C$40*1000</f>
+        <f>Calculations!U67-About!$C$47*1000</f>
         <v>19112.986661782561</v>
       </c>
       <c r="T8">
-        <f>Calculations!V67-About!$C$40*1000</f>
+        <f>Calculations!V67-About!$C$47*1000</f>
         <v>20148.406524245118</v>
       </c>
       <c r="U8">
-        <f>Calculations!W67-About!$C$40*1000</f>
+        <f>Calculations!W67-About!$C$47*1000</f>
         <v>21216.417810491377</v>
       </c>
       <c r="V8">
-        <f>Calculations!X67-About!$C$40*1000</f>
+        <f>Calculations!X67-About!$C$47*1000</f>
         <v>22326.006050190234</v>
       </c>
       <c r="W8">
-        <f>Calculations!Y67-About!$C$40*1000</f>
+        <f>Calculations!Y67-About!$C$47*1000</f>
         <v>23463.187522140372</v>
       </c>
       <c r="X8">
-        <f>Calculations!Z67-About!$C$40*1000</f>
+        <f>Calculations!Z67-About!$C$47*1000</f>
         <v>24635.09109795191</v>
       </c>
       <c r="Y8">
-        <f>Calculations!AA67-About!$C$40*1000</f>
+        <f>Calculations!AA67-About!$C$47*1000</f>
         <v>25843.173991580989</v>
       </c>
       <c r="Z8">
-        <f>Calculations!AB67-About!$C$40*1000</f>
+        <f>Calculations!AB67-About!$C$47*1000</f>
         <v>27104.401081923417</v>
       </c>
       <c r="AA8">
-        <f>Calculations!AC67-About!$C$40*1000</f>
+        <f>Calculations!AC67-About!$C$47*1000</f>
         <v>28388.887146280256</v>
       </c>
       <c r="AB8">
-        <f>Calculations!AD67-About!$C$40*1000</f>
+        <f>Calculations!AD67-About!$C$47*1000</f>
         <v>29719.572463207314</v>
       </c>
     </row>
@@ -28286,7 +29283,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -28587,113 +29584,113 @@
       <c r="A4" t="s">
         <v>600</v>
       </c>
-      <c r="B4">
-        <f>Calculations!D84</f>
-        <v>1468.7250000000001</v>
-      </c>
-      <c r="C4">
-        <f>Calculations!E84</f>
-        <v>1508.008</v>
-      </c>
-      <c r="D4">
-        <f>Calculations!F84</f>
-        <v>1540.9690000000001</v>
-      </c>
-      <c r="E4">
-        <f>Calculations!G84</f>
-        <v>1559.125</v>
-      </c>
-      <c r="F4">
-        <f>Calculations!H84</f>
-        <v>1576.8690000000001</v>
-      </c>
-      <c r="G4">
-        <f>Calculations!I84</f>
-        <v>1595.395</v>
-      </c>
-      <c r="H4">
-        <f>Calculations!J84</f>
-        <v>1615.2909999999999</v>
-      </c>
-      <c r="I4">
-        <f>Calculations!K84</f>
-        <v>1634.761</v>
-      </c>
-      <c r="J4">
-        <f>Calculations!L84</f>
-        <v>1655.3439999999998</v>
-      </c>
-      <c r="K4">
-        <f>Calculations!M84</f>
-        <v>1676.5520000000001</v>
-      </c>
-      <c r="L4">
-        <f>Calculations!N84</f>
-        <v>1700.0949999999998</v>
-      </c>
-      <c r="M4">
-        <f>Calculations!O84</f>
-        <v>1722.0139999999999</v>
-      </c>
-      <c r="N4">
-        <f>Calculations!P84</f>
-        <v>1744.8120000000001</v>
-      </c>
-      <c r="O4">
-        <f>Calculations!Q84</f>
-        <v>1769.9970000000001</v>
-      </c>
-      <c r="P4">
-        <f>Calculations!R84</f>
-        <v>1793.4589999999998</v>
-      </c>
-      <c r="Q4">
-        <f>Calculations!S84</f>
-        <v>1816.316</v>
-      </c>
-      <c r="R4">
-        <f>Calculations!T84</f>
-        <v>1838.2280000000001</v>
-      </c>
-      <c r="S4">
-        <f>Calculations!U84</f>
-        <v>1858.4989999999998</v>
-      </c>
-      <c r="T4">
-        <f>Calculations!V84</f>
-        <v>1881.0849999999998</v>
-      </c>
-      <c r="U4">
-        <f>Calculations!W84</f>
-        <v>1901.162</v>
-      </c>
-      <c r="V4">
-        <f>Calculations!X84</f>
-        <v>1921.1780000000001</v>
-      </c>
-      <c r="W4">
-        <f>Calculations!Y84</f>
-        <v>1940.0839999999998</v>
-      </c>
-      <c r="X4">
-        <f>Calculations!Z84</f>
-        <v>1959.433</v>
-      </c>
-      <c r="Y4">
-        <f>Calculations!AA84</f>
-        <v>1979.941</v>
-      </c>
-      <c r="Z4">
-        <f>Calculations!AB84</f>
-        <v>2000.0969999999998</v>
-      </c>
-      <c r="AA4">
-        <f>Calculations!AC84</f>
-        <v>2019.018</v>
-      </c>
-      <c r="AB4">
-        <f>Calculations!AD84</f>
-        <v>2039.0600000000002</v>
+      <c r="B4" s="64">
+        <f>'Data Center Gas'!C27</f>
+        <v>13468.725</v>
+      </c>
+      <c r="C4" s="64">
+        <f>'Data Center Gas'!D27</f>
+        <v>18508.008000000002</v>
+      </c>
+      <c r="D4" s="64">
+        <f>'Data Center Gas'!E27</f>
+        <v>22540.969000000001</v>
+      </c>
+      <c r="E4" s="64">
+        <f>'Data Center Gas'!F27</f>
+        <v>26559.125</v>
+      </c>
+      <c r="F4" s="64">
+        <f>'Data Center Gas'!G27</f>
+        <v>30576.868999999999</v>
+      </c>
+      <c r="G4" s="64">
+        <f>'Data Center Gas'!H27</f>
+        <v>40595.394999999997</v>
+      </c>
+      <c r="H4" s="64">
+        <f>'Data Center Gas'!I27</f>
+        <v>50615.290999999997</v>
+      </c>
+      <c r="I4" s="64">
+        <f>'Data Center Gas'!J27</f>
+        <v>50634.760999999999</v>
+      </c>
+      <c r="J4" s="64">
+        <f>'Data Center Gas'!K27</f>
+        <v>50655.343999999997</v>
+      </c>
+      <c r="K4" s="64">
+        <f>'Data Center Gas'!L27</f>
+        <v>50676.552000000003</v>
+      </c>
+      <c r="L4" s="64">
+        <f>'Data Center Gas'!M27</f>
+        <v>50700.095000000001</v>
+      </c>
+      <c r="M4" s="64">
+        <f>'Data Center Gas'!N27</f>
+        <v>50722.014000000003</v>
+      </c>
+      <c r="N4" s="64">
+        <f>'Data Center Gas'!O27</f>
+        <v>50744.811999999998</v>
+      </c>
+      <c r="O4" s="64">
+        <f>'Data Center Gas'!P27</f>
+        <v>50769.997000000003</v>
+      </c>
+      <c r="P4" s="64">
+        <f>'Data Center Gas'!Q27</f>
+        <v>50793.459000000003</v>
+      </c>
+      <c r="Q4" s="64">
+        <f>'Data Center Gas'!R27</f>
+        <v>50816.315999999999</v>
+      </c>
+      <c r="R4" s="64">
+        <f>'Data Center Gas'!S27</f>
+        <v>50838.228000000003</v>
+      </c>
+      <c r="S4" s="64">
+        <f>'Data Center Gas'!T27</f>
+        <v>50858.498999999996</v>
+      </c>
+      <c r="T4" s="64">
+        <f>'Data Center Gas'!U27</f>
+        <v>50881.084999999999</v>
+      </c>
+      <c r="U4" s="64">
+        <f>'Data Center Gas'!V27</f>
+        <v>50901.161999999997</v>
+      </c>
+      <c r="V4" s="64">
+        <f>'Data Center Gas'!W27</f>
+        <v>50921.178</v>
+      </c>
+      <c r="W4" s="64">
+        <f>'Data Center Gas'!X27</f>
+        <v>50940.084000000003</v>
+      </c>
+      <c r="X4" s="64">
+        <f>'Data Center Gas'!Y27</f>
+        <v>50959.432999999997</v>
+      </c>
+      <c r="Y4" s="64">
+        <f>'Data Center Gas'!Z27</f>
+        <v>50979.940999999999</v>
+      </c>
+      <c r="Z4" s="64">
+        <f>'Data Center Gas'!AA27</f>
+        <v>51000.097000000002</v>
+      </c>
+      <c r="AA4" s="64">
+        <f>'Data Center Gas'!AB27</f>
+        <v>51019.017999999996</v>
+      </c>
+      <c r="AB4" s="64">
+        <f>'Data Center Gas'!AC27</f>
+        <v>51039.06</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
@@ -29040,111 +30037,111 @@
         <v>535</v>
       </c>
       <c r="B8">
-        <f>Calculations!D88-About!$C$36*1000</f>
+        <f>Calculations!D88-About!$C$43*1000</f>
         <v>21769.497000000003</v>
       </c>
       <c r="C8">
-        <f>Calculations!E88-About!$C$36*1000</f>
+        <f>Calculations!E88-About!$C$43*1000</f>
         <v>25925.201999999997</v>
       </c>
       <c r="D8">
-        <f>Calculations!F88-About!$C$36*1000</f>
+        <f>Calculations!F88-About!$C$43*1000</f>
         <v>30160.527000000002</v>
       </c>
       <c r="E8">
-        <f>Calculations!G88-About!$C$36*1000</f>
+        <f>Calculations!G88-About!$C$43*1000</f>
         <v>33771.183000000005</v>
       </c>
       <c r="F8">
-        <f>Calculations!H88-About!$C$36*1000</f>
+        <f>Calculations!H88-About!$C$43*1000</f>
         <v>35511.208000000006</v>
       </c>
       <c r="G8">
-        <f>Calculations!I88-About!$C$36*1000</f>
+        <f>Calculations!I88-About!$C$43*1000</f>
         <v>36631.794000000002</v>
       </c>
       <c r="H8">
-        <f>Calculations!J88-About!$C$36*1000</f>
+        <f>Calculations!J88-About!$C$43*1000</f>
         <v>37899.681000000004</v>
       </c>
       <c r="I8">
-        <f>Calculations!K88-About!$C$36*1000</f>
+        <f>Calculations!K88-About!$C$43*1000</f>
         <v>38829.173999999999</v>
       </c>
       <c r="J8">
-        <f>Calculations!L88-About!$C$36*1000</f>
+        <f>Calculations!L88-About!$C$43*1000</f>
         <v>39576.554000000004</v>
       </c>
       <c r="K8">
-        <f>Calculations!M88-About!$C$36*1000</f>
+        <f>Calculations!M88-About!$C$43*1000</f>
         <v>40414.337000000007</v>
       </c>
       <c r="L8">
-        <f>Calculations!N88-About!$C$36*1000</f>
+        <f>Calculations!N88-About!$C$43*1000</f>
         <v>41719.628000000004</v>
       </c>
       <c r="M8">
-        <f>Calculations!O88-About!$C$36*1000</f>
+        <f>Calculations!O88-About!$C$43*1000</f>
         <v>42791.535000000003</v>
       </c>
       <c r="N8">
-        <f>Calculations!P88-About!$C$36*1000</f>
+        <f>Calculations!P88-About!$C$43*1000</f>
         <v>43690.09</v>
       </c>
       <c r="O8">
-        <f>Calculations!Q88-About!$C$36*1000</f>
+        <f>Calculations!Q88-About!$C$43*1000</f>
         <v>45293.167000000001</v>
       </c>
       <c r="P8">
-        <f>Calculations!R88-About!$C$36*1000</f>
+        <f>Calculations!R88-About!$C$43*1000</f>
         <v>46843.823000000004</v>
       </c>
       <c r="Q8">
-        <f>Calculations!S88-About!$C$36*1000</f>
+        <f>Calculations!S88-About!$C$43*1000</f>
         <v>48761.62</v>
       </c>
       <c r="R8">
-        <f>Calculations!T88-About!$C$36*1000</f>
+        <f>Calculations!T88-About!$C$43*1000</f>
         <v>50386.563000000002</v>
       </c>
       <c r="S8">
-        <f>Calculations!U88-About!$C$36*1000</f>
+        <f>Calculations!U88-About!$C$43*1000</f>
         <v>51249.068999999996</v>
       </c>
       <c r="T8">
-        <f>Calculations!V88-About!$C$36*1000</f>
+        <f>Calculations!V88-About!$C$43*1000</f>
         <v>52600.880000000005</v>
       </c>
       <c r="U8">
-        <f>Calculations!W88-About!$C$36*1000</f>
+        <f>Calculations!W88-About!$C$43*1000</f>
         <v>53315.83</v>
       </c>
       <c r="V8">
-        <f>Calculations!X88-About!$C$36*1000</f>
+        <f>Calculations!X88-About!$C$43*1000</f>
         <v>54131.939000000006</v>
       </c>
       <c r="W8">
-        <f>Calculations!Y88-About!$C$36*1000</f>
+        <f>Calculations!Y88-About!$C$43*1000</f>
         <v>54786.152000000002</v>
       </c>
       <c r="X8">
-        <f>Calculations!Z88-About!$C$36*1000</f>
+        <f>Calculations!Z88-About!$C$43*1000</f>
         <v>55810.433000000005</v>
       </c>
       <c r="Y8">
-        <f>Calculations!AA88-About!$C$36*1000</f>
+        <f>Calculations!AA88-About!$C$43*1000</f>
         <v>57088.451999999997</v>
       </c>
       <c r="Z8">
-        <f>Calculations!AB88-About!$C$36*1000</f>
+        <f>Calculations!AB88-About!$C$43*1000</f>
         <v>58391.651000000005</v>
       </c>
       <c r="AA8">
-        <f>Calculations!AC88-About!$C$36*1000</f>
+        <f>Calculations!AC88-About!$C$43*1000</f>
         <v>59345.417000000009</v>
       </c>
       <c r="AB8">
-        <f>Calculations!AD88-About!$C$36*1000</f>
+        <f>Calculations!AD88-About!$C$43*1000</f>
         <v>60616.367999999995</v>
       </c>
     </row>
@@ -30885,8 +31882,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB692F98-9304-4C26-AFDF-8AB624EA8082}">
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6312F16-2538-4421-91BC-5D10BE5A5338}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
@@ -30900,13 +31897,13 @@
       <c r="A1" t="s">
         <v>548</v>
       </c>
-      <c r="B1" s="79" t="s">
-        <v>977</v>
-      </c>
-      <c r="C1" s="79" t="s">
-        <v>978</v>
-      </c>
-      <c r="D1" s="79" t="s">
+      <c r="B1" s="96" t="s">
+        <v>998</v>
+      </c>
+      <c r="C1" s="96" t="s">
+        <v>999</v>
+      </c>
+      <c r="D1" s="96" t="s">
         <v>973</v>
       </c>
     </row>
@@ -30948,9 +31945,9 @@
       <c r="C4">
         <v>0</v>
       </c>
-      <c r="D4" s="80">
+      <c r="D4" s="97">
         <f>'BDESC-commercial'!B4</f>
-        <v>1468.7250000000001</v>
+        <v>13468.725</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -30985,15 +31982,15 @@
       <c r="A7" t="s">
         <v>533</v>
       </c>
-      <c r="B7" s="80">
+      <c r="B7" s="97">
         <f>'BDESC-urban-residential'!B7</f>
         <v>250.57474912976602</v>
       </c>
-      <c r="C7" s="80">
+      <c r="C7" s="97">
         <f>'BDESC-rural-residential'!B7</f>
         <v>57.60425087023394</v>
       </c>
-      <c r="D7" s="80">
+      <c r="D7" s="97">
         <f>'BDESC-commercial'!B7</f>
         <v>585.6400000000001</v>
       </c>
@@ -31002,15 +31999,15 @@
       <c r="A8" t="s">
         <v>535</v>
       </c>
-      <c r="B8" s="81">
+      <c r="B8" s="98">
         <f>'BDESC-urban-residential'!B8</f>
         <v>30362.289170242049</v>
       </c>
-      <c r="C8" s="80">
+      <c r="C8" s="97">
         <f>'BDESC-rural-residential'!B8</f>
         <v>6979.940829757953</v>
       </c>
-      <c r="D8" s="80">
+      <c r="D8" s="97">
         <f>'BDESC-commercial'!B8</f>
         <v>21769.497000000003</v>
       </c>
@@ -31067,7 +32064,7 @@
       <c r="C12">
         <v>0</v>
       </c>
-      <c r="D12" s="80">
+      <c r="D12" s="97">
         <f>'BDESC-commercial'!B12</f>
         <v>20.507000000000001</v>
       </c>
@@ -31274,105 +32271,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="73" t="s">
         <v>958</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="67"/>
-      <c r="S1" s="67"/>
-      <c r="T1" s="67"/>
-      <c r="U1" s="67"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
     </row>
     <row r="2" spans="1:21" ht="39" x14ac:dyDescent="0.25">
       <c r="A2" s="63" t="s">
         <v>957</v>
       </c>
-      <c r="B2" s="64" t="s">
+      <c r="B2" s="74" t="s">
         <v>956</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="65"/>
-      <c r="P2" s="64" t="s">
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="76"/>
+      <c r="P2" s="74" t="s">
         <v>955</v>
       </c>
-      <c r="Q2" s="65"/>
-      <c r="R2" s="64" t="s">
+      <c r="Q2" s="76"/>
+      <c r="R2" s="74" t="s">
         <v>954</v>
       </c>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
-      <c r="U2" s="65"/>
+      <c r="S2" s="75"/>
+      <c r="T2" s="75"/>
+      <c r="U2" s="76"/>
     </row>
     <row r="3" spans="1:21" ht="39" x14ac:dyDescent="0.25">
       <c r="A3" s="63" t="s">
         <v>953</v>
       </c>
-      <c r="B3" s="64" t="s">
+      <c r="B3" s="74" t="s">
         <v>85</v>
       </c>
-      <c r="C3" s="65"/>
-      <c r="D3" s="64" t="s">
+      <c r="C3" s="76"/>
+      <c r="D3" s="74" t="s">
         <v>952</v>
       </c>
-      <c r="E3" s="65"/>
-      <c r="F3" s="64" t="s">
+      <c r="E3" s="76"/>
+      <c r="F3" s="74" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="65"/>
-      <c r="H3" s="64" t="s">
+      <c r="G3" s="76"/>
+      <c r="H3" s="74" t="s">
         <v>951</v>
       </c>
-      <c r="I3" s="65"/>
-      <c r="J3" s="64" t="s">
+      <c r="I3" s="76"/>
+      <c r="J3" s="74" t="s">
         <v>950</v>
       </c>
-      <c r="K3" s="65"/>
-      <c r="L3" s="64" t="s">
+      <c r="K3" s="76"/>
+      <c r="L3" s="74" t="s">
         <v>949</v>
       </c>
-      <c r="M3" s="65"/>
-      <c r="N3" s="64" t="s">
+      <c r="M3" s="76"/>
+      <c r="N3" s="74" t="s">
         <v>948</v>
       </c>
-      <c r="O3" s="65"/>
-      <c r="P3" s="64" t="s">
+      <c r="O3" s="76"/>
+      <c r="P3" s="74" t="s">
         <v>947</v>
       </c>
-      <c r="Q3" s="65"/>
-      <c r="R3" s="64" t="s">
+      <c r="Q3" s="76"/>
+      <c r="R3" s="74" t="s">
         <v>946</v>
       </c>
-      <c r="S3" s="65"/>
-      <c r="T3" s="64" t="s">
+      <c r="S3" s="76"/>
+      <c r="T3" s="74" t="s">
         <v>945</v>
       </c>
-      <c r="U3" s="65"/>
+      <c r="U3" s="76"/>
     </row>
     <row r="4" spans="1:21" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A4" s="63" t="s">
@@ -35470,32 +36467,33 @@
       </c>
     </row>
     <row r="67" spans="1:21" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="66" t="s">
+      <c r="A67" s="72" t="s">
         <v>886</v>
       </c>
-      <c r="B67" s="66"/>
-      <c r="C67" s="66"/>
-      <c r="D67" s="66"/>
-      <c r="E67" s="66"/>
-      <c r="F67" s="66"/>
-      <c r="G67" s="66"/>
-      <c r="H67" s="66"/>
-      <c r="I67" s="66"/>
-      <c r="J67" s="66"/>
-      <c r="K67" s="66"/>
-      <c r="L67" s="66"/>
-      <c r="M67" s="66"/>
-      <c r="N67" s="66"/>
-      <c r="O67" s="66"/>
-      <c r="P67" s="66"/>
-      <c r="Q67" s="66"/>
-      <c r="R67" s="66"/>
-      <c r="S67" s="66"/>
-      <c r="T67" s="66"/>
-      <c r="U67" s="66"/>
+      <c r="B67" s="72"/>
+      <c r="C67" s="72"/>
+      <c r="D67" s="72"/>
+      <c r="E67" s="72"/>
+      <c r="F67" s="72"/>
+      <c r="G67" s="72"/>
+      <c r="H67" s="72"/>
+      <c r="I67" s="72"/>
+      <c r="J67" s="72"/>
+      <c r="K67" s="72"/>
+      <c r="L67" s="72"/>
+      <c r="M67" s="72"/>
+      <c r="N67" s="72"/>
+      <c r="O67" s="72"/>
+      <c r="P67" s="72"/>
+      <c r="Q67" s="72"/>
+      <c r="R67" s="72"/>
+      <c r="S67" s="72"/>
+      <c r="T67" s="72"/>
+      <c r="U67" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A67:U67"/>
     <mergeCell ref="A1:U1"/>
     <mergeCell ref="B2:O2"/>
     <mergeCell ref="P2:Q2"/>
@@ -35510,7 +36508,6 @@
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="R3:S3"/>
     <mergeCell ref="T3:U3"/>
-    <mergeCell ref="A67:U67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup scale="37" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -48207,43 +49204,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="86" t="s">
         <v>368</v>
       </c>
-      <c r="B1" s="75"/>
+      <c r="B1" s="83"/>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="82" t="s">
         <v>369</v>
       </c>
-      <c r="B2" s="75"/>
-      <c r="C2" s="75"/>
-      <c r="D2" s="75"/>
-      <c r="E2" s="75"/>
-      <c r="F2" s="75"/>
-      <c r="G2" s="75"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
     </row>
     <row r="3" spans="1:7" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
-      <c r="B3" s="69" t="s">
+      <c r="B3" s="77" t="s">
         <v>370</v>
       </c>
-      <c r="C3" s="70"/>
-      <c r="D3" s="70"/>
-      <c r="E3" s="70"/>
-      <c r="F3" s="70"/>
-      <c r="G3" s="70"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
     </row>
     <row r="4" spans="1:7" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17"/>
       <c r="B4" s="19"/>
-      <c r="C4" s="71" t="s">
+      <c r="C4" s="79" t="s">
         <v>371</v>
       </c>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="73"/>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="81"/>
     </row>
     <row r="5" spans="1:7" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20"/>
@@ -52764,15 +53761,15 @@
       <c r="G220" s="25"/>
     </row>
     <row r="221" spans="1:7" s="6" customFormat="1" ht="206.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A221" s="76" t="s">
+      <c r="A221" s="84" t="s">
         <v>522</v>
       </c>
-      <c r="B221" s="77"/>
-      <c r="C221" s="77"/>
-      <c r="D221" s="77"/>
-      <c r="E221" s="77"/>
-      <c r="F221" s="77"/>
-      <c r="G221" s="77"/>
+      <c r="B221" s="85"/>
+      <c r="C221" s="85"/>
+      <c r="D221" s="85"/>
+      <c r="E221" s="85"/>
+      <c r="F221" s="85"/>
+      <c r="G221" s="85"/>
     </row>
     <row r="222" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>